<commit_message>
To work on it during the holiday
</commit_message>
<xml_diff>
--- a/DBs/Lander state of the art.xlsx
+++ b/DBs/Lander state of the art.xlsx
@@ -1,25 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdepaor2\Desktop\ORLA ACTA Paper\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdepaor2\Desktop\ORLA_Lander_Mission_Architecture\DBs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D9B3893-96A1-4578-9CF7-0FCD06B88128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8D700E-BB37-4BA9-9D81-994005CEABE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9B8D5217-16A3-40F0-9DB1-748038C9A303}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{9B8D5217-16A3-40F0-9DB1-748038C9A303}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Feuil1!$H$19</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Feuil1!$B$3:$B$15</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Feuil1!$E$3</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Feuil1!$H$19</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Feuil1!$B$3:$B$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -218,19 +215,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -1383,7 +1375,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2637,14 +2629,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2682,7 +2670,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2788,7 +2776,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2930,7 +2918,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2938,7 +2926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9D55D17-879F-4BD2-AFB3-F96D608713F1}">
-  <dimension ref="B2:H22"/>
+  <dimension ref="B2:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.140625" customWidth="1"/>
@@ -2950,347 +2938,326 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>2024</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>3200</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="1">
         <v>700</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>2024</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>710</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="1">
         <v>20</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>120</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>2024</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>1283</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="1">
         <v>90</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>2024</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>1908</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="1">
         <v>100</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>118</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>2023</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>1750</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="1">
         <v>30</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="1">
         <v>135</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>2023</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>1000</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="1">
         <v>30</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>2023</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>1750</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="1">
         <v>26</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="1">
         <v>72</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>2022</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>14.6</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="1">
         <v>0.1</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>6</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>2020</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>3800</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="1">
         <v>800</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>2019</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>1471</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="1">
         <v>27</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>115</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>2019</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>3640</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="1">
         <v>170</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>2019</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>585</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="1">
         <v>0.1</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>100</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>2013</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>3780</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="1">
         <v>170</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="H15" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H19" s="6"/>
-    </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H21" s="6"/>
-    </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H22" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>